<commit_message>
fix excel import files
</commit_message>
<xml_diff>
--- a/public/excel/customer-import-sample.xlsx
+++ b/public/excel/customer-import-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>first_name</t>
   </si>
@@ -31,6 +31,12 @@
     <t>gender</t>
   </si>
   <si>
+    <t>license_no</t>
+  </si>
+  <si>
+    <t>license_verified</t>
+  </si>
+  <si>
     <t>Test</t>
   </si>
   <si>
@@ -47,7 +53,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -57,6 +63,11 @@
     <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -73,11 +84,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -316,25 +330,37 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2">
-        <v>8.80123456789E11</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="C2" s="3">
+        <v>3.30123456789E11</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>10</v>
       </c>
       <c r="E2" s="1">
         <v>123456.0</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1.1111111111111E13</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1.0</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1"/>

</xml_diff>